<commit_message>
status: revision part 1
</commit_message>
<xml_diff>
--- a/manuscript/revision/reviewer-comments.xlsx
+++ b/manuscript/revision/reviewer-comments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/toby/Desktop/Repositories/ankle-draft-II/manuscript/revision/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C8240F9-DA27-6C4E-9C0E-715C54B57966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F1BD3D5-0556-434E-9395-BDCA17574634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2740" yWindow="1060" windowWidth="34200" windowHeight="19920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reviewer Comments" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="83">
   <si>
     <t>ID</t>
   </si>
@@ -191,13 +191,91 @@
   </si>
   <si>
     <t>Response</t>
+  </si>
+  <si>
+    <t>Comments Stefano</t>
+  </si>
+  <si>
+    <t>If not already there, we can add it based on previous results.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">we knew this was a concern. We should underline in the answer that we used the ABC model (we may tell a bit more about why it is good and what it is) to predict what would have happened with a longer exposure. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">If not reported, we should add it and check it but not differenciate models based on sex because it may not applicable in standards. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">We should not only focus on downdraft, but our model is also generic. It should also be applicable to floor diffusers. Nevertheless, a deeper explanation of how we selected the tested conditions would be valuable. </t>
+  </si>
+  <si>
+    <t>we already did it, so we should point it out in the answer to the reviewer. Worth adding a reference to previous papers (both us and others, including the draft risk model of the past - Fanger/Melikov) and the fact that ASHRAE 55 asks to evaluate a condition for a 15 min.</t>
+  </si>
+  <si>
+    <t>yes, this is the aim of the model.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ok to do in the paper, we will not do it in the addenda. </t>
+  </si>
+  <si>
+    <t>Done?</t>
+  </si>
+  <si>
+    <t>Suggestion</t>
+  </si>
+  <si>
+    <t>AGREE</t>
+  </si>
+  <si>
+    <t>POTENTIAL REFUTE</t>
+  </si>
+  <si>
+    <t>DONE</t>
+  </si>
+  <si>
+    <t>The first highlight has been adjusted to be within the character limit.</t>
+  </si>
+  <si>
+    <t>The graphical abstract has been adjusted to correct this error.</t>
+  </si>
+  <si>
+    <t>The number has been corrected to reflect the most up-to-date value from the analysis covered in the Results section.</t>
+  </si>
+  <si>
+    <t>The abstract has been adjusted to include information about these limitations.</t>
+  </si>
+  <si>
+    <t>Confirm updated abstract with Stefano.</t>
+  </si>
+  <si>
+    <t>This has been corrected and values are now shown as percentage values in the table.</t>
+  </si>
+  <si>
+    <t>This error has been pointed out correctly. The actual value changed to 30% (after updating the analysis). The values are now consistent across the paper.</t>
+  </si>
+  <si>
+    <t>PATRICK</t>
+  </si>
+  <si>
+    <t>The correct value of 0.6 clo is now used throughout the paper.</t>
+  </si>
+  <si>
+    <t>Thanks for pointing this out. The sentence is now completed.</t>
+  </si>
+  <si>
+    <t>The figures have been created using the minimum font size in B&amp;E author guidelines (7pt) and with typical column widths in mind. In the manuscript submitted as a Word document, they are not shown at full width, meaning that fonts appear smaller than they would in the actual paper. Nonetheless, we have increased the minimum font size for most figures to 8pt to enhance clarity and readability.</t>
+  </si>
+  <si>
+    <t>Patrick to review his figures, too. For example skin temperature figures.</t>
+  </si>
+  <si>
+    <t>The axes have been removed on purpose for aesthetic reasons. But we agree with the second comment about the R² labels and have adjusted the figure legends accordingly to make this clearer.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -210,21 +288,32 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -249,6 +338,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEDF7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -279,7 +392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -302,7 +415,34 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -607,16 +747,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="100" customWidth="1"/>
-    <col min="4" max="4" width="28.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.33203125" style="14" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="80.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -626,11 +770,23 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -640,8 +796,18 @@
       <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D2" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" s="8"/>
+    </row>
+    <row r="3" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -651,8 +817,20 @@
       <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D3" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>8</v>
       </c>
@@ -662,8 +840,17 @@
       <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D4" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="8"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -673,8 +860,20 @@
       <c r="C5" s="5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D5" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
@@ -684,8 +883,14 @@
       <c r="C6" s="5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D6" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="8"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="8"/>
+    </row>
+    <row r="7" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>15</v>
       </c>
@@ -695,8 +900,14 @@
       <c r="C7" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D7" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="8"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="8"/>
+    </row>
+    <row r="8" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
@@ -706,8 +917,18 @@
       <c r="C8" s="5" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D8" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="G8" s="8"/>
+    </row>
+    <row r="9" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>19</v>
       </c>
@@ -717,8 +938,14 @@
       <c r="C9" s="5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D9" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" s="8"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="8"/>
+    </row>
+    <row r="10" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>21</v>
       </c>
@@ -728,8 +955,17 @@
       <c r="C10" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D10" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="8"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>23</v>
       </c>
@@ -739,8 +975,14 @@
       <c r="C11" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D11" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="8"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="8"/>
+    </row>
+    <row r="12" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>25</v>
       </c>
@@ -750,8 +992,18 @@
       <c r="C12" s="5" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D12" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" s="15"/>
+    </row>
+    <row r="13" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>27</v>
       </c>
@@ -761,8 +1013,18 @@
       <c r="C13" s="5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D13" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" s="8"/>
+    </row>
+    <row r="14" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>29</v>
       </c>
@@ -772,8 +1034,16 @@
       <c r="C14" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D14" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" s="9"/>
+      <c r="G14" s="8"/>
+    </row>
+    <row r="15" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>31</v>
       </c>
@@ -783,8 +1053,18 @@
       <c r="C15" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D15" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="G15" s="8"/>
+    </row>
+    <row r="16" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>33</v>
       </c>
@@ -794,8 +1074,16 @@
       <c r="C16" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D16" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" s="9"/>
+      <c r="G16" s="8"/>
+    </row>
+    <row r="17" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>35</v>
       </c>
@@ -805,8 +1093,19 @@
       <c r="C17" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D17" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="9"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>37</v>
       </c>
@@ -816,8 +1115,19 @@
       <c r="C18" s="5" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D18" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="G18" s="8"/>
+      <c r="H18" s="9"/>
+    </row>
+    <row r="19" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>39</v>
       </c>
@@ -827,8 +1137,19 @@
       <c r="C19" s="5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D19" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="G19" s="8"/>
+      <c r="H19" s="9"/>
+    </row>
+    <row r="20" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
         <v>41</v>
       </c>
@@ -838,8 +1159,17 @@
       <c r="C20" s="7" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D20" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="8"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
         <v>44</v>
       </c>
@@ -849,8 +1179,15 @@
       <c r="C21" s="7" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D21" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="8"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="9"/>
+    </row>
+    <row r="22" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>46</v>
       </c>
@@ -860,8 +1197,17 @@
       <c r="C22" s="7" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D22" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" s="8"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
         <v>48</v>
       </c>
@@ -871,8 +1217,19 @@
       <c r="C23" s="7" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D23" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="G23" s="8"/>
+      <c r="H23" s="9"/>
+    </row>
+    <row r="24" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
         <v>50</v>
       </c>
@@ -882,8 +1239,16 @@
       <c r="C24" s="7" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D24" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24" s="9"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
         <v>52</v>
       </c>
@@ -893,8 +1258,19 @@
       <c r="C25" s="7" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D25" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="F25" s="9"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
         <v>54</v>
       </c>
@@ -904,6 +1280,13 @@
       <c r="C26" s="7" t="s">
         <v>55</v>
       </c>
+      <c r="D26" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E26" s="8"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
status: before power analysis
</commit_message>
<xml_diff>
--- a/manuscript/revision/reviewer-comments.xlsx
+++ b/manuscript/revision/reviewer-comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/toby/Desktop/Repositories/ankle-draft-II/manuscript/revision/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F1BD3D5-0556-434E-9395-BDCA17574634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9F266B-0BDD-3A4D-8089-8767F060B473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2740" yWindow="1060" windowWidth="34200" windowHeight="19920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="90">
   <si>
     <t>ID</t>
   </si>
@@ -269,13 +269,35 @@
   </si>
   <si>
     <t>The axes have been removed on purpose for aesthetic reasons. But we agree with the second comment about the R² labels and have adjusted the figure legends accordingly to make this clearer.</t>
+  </si>
+  <si>
+    <t>We would like to clarify that the LME fits in Section 3.2 are descriptive visualizations; the detailed inferential predictor analysis, including p-values, is presented in Table 4. Here we report R² as the effect size, with reference based Ferguson (2009).</t>
+  </si>
+  <si>
+    <t>Confirm with Patrick</t>
+  </si>
+  <si>
+    <t>We thank the reviewer for raising this point. We note that clothing insulation (clo) is a whole-body ensemble property defined for global thermal balance calculations; it cannot be directly disaggregated into standardized region-specific values. Consequently, a 'local clo for the ankle region' is not a quantity defined or utilized in ASHRAE 55 or ISO 9920. More broadly, the 0.75 clo figure serves strictly to characterize the experimental clothing scenario relative to prior work and it is not an input parameter for the ankle draft model, which relies on local air speed, local air temperature, and whole-body thermal sensation as predictors. The protective effect of the clothing is already captured empirically through the measured skin temperatures and subjective comfort votes.</t>
+  </si>
+  <si>
+    <t>Confirm with team.</t>
+  </si>
+  <si>
+    <t>We agree with this comment. We have renamed all instances of 'ankle skin temperature' to 'lower-leg skin temperature' throughout Section 3.3.3 and the associated figure captions to accurately reflect the measurement locations (mid-calf and dorsum of the foot). We have also added a clarifying sentence to the Physiological Monitoring section of the Methods explaining that these sites were chosen as the most practical iButton attachment locations bracketing the ankle region, and that direct placement at the ankle was not feasible due to the ankle bone.</t>
+  </si>
+  <si>
+    <t>We respectfully note that ankle-level air temperature and air speed across the three seated positions are already reported in Table 3, which presents measured values (mean ± SD) separately for each workstation (low, medium, high air speed) across all three session temperature conditions. The consistency of local conditions across positions is evident from the low standard deviations reported there.</t>
+  </si>
+  <si>
+    <t>We thank the reviewer for raising this point. The 20-minute exposure was chosen deliberately to match the duration used in the foundational ankle draft studies by Liu et al. (2017) and Schiavon et al. (2016), enabling direct comparability. This duration is also consistent with the broader local thermal discomfort literature and exceeds the 15-minute evaluation window specified in ASHRAE Standard 55 for assessing local discomfort conditions.
+To assess the potential effect of longer exposure, we extrapolated the measured lower-leg skin temperature trajectories to 90 minutes using exponential models, and validated these projections against the Advanced Berkeley Comfort (ABC) model, a multi-node transient human thermal model that simulates heat exchange between body segments and the environment over time and has been extensively validated against experimental data (Huizenga et al., 2001). The ABC model predicted an additional lower-leg skin temperature decrease of only 0.3–0.7°C beyond 20 minutes and a corresponding change in whole-body thermal sensation below 0.3 TSV units. We acknowledge that subjective dissatisfaction rates beyond the tested period cannot be directly predicted and may be somewhat higher under sustained exposure; this is discussed in the Limitations section and the relevant passage in the Results has been revised to reflect this uncertainty more explicitly.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,6 +330,13 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.249977111117893"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -392,7 +421,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -443,6 +472,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -886,9 +921,15 @@
       <c r="D6" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="E6" s="8"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="8"/>
+      <c r="E6" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
@@ -903,8 +944,12 @@
       <c r="D7" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="8"/>
-      <c r="F7" s="9"/>
+      <c r="E7" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>87</v>
+      </c>
       <c r="G7" s="8"/>
     </row>
     <row r="8" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -941,9 +986,15 @@
       <c r="D9" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="8"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="8"/>
+      <c r="E9" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
@@ -958,8 +1009,12 @@
       <c r="D10" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="E10" s="8"/>
-      <c r="F10" s="9"/>
+      <c r="E10" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>89</v>
+      </c>
       <c r="G10" s="8"/>
       <c r="H10" s="9" t="s">
         <v>59</v>
@@ -1179,11 +1234,15 @@
       <c r="C21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D21" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21" s="8"/>
-      <c r="F21" s="9"/>
+      <c r="D21" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="E21" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>88</v>
+      </c>
       <c r="G21" s="8"/>
       <c r="H21" s="9"/>
     </row>

</xml_diff>

<commit_message>
fix: remove redundant files
</commit_message>
<xml_diff>
--- a/manuscript/revision/reviewer-comments.xlsx
+++ b/manuscript/revision/reviewer-comments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/toby/Desktop/Repositories/ankle-draft-II/manuscript/revision/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9F266B-0BDD-3A4D-8089-8767F060B473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3A3B473-6A4F-A448-9A69-99113FC4457F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2740" yWindow="1060" windowWidth="34200" windowHeight="19920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-380" yWindow="840" windowWidth="34200" windowHeight="19920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reviewer Comments" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="97">
   <si>
     <t>ID</t>
   </si>
@@ -291,6 +291,27 @@
   <si>
     <t>We thank the reviewer for raising this point. The 20-minute exposure was chosen deliberately to match the duration used in the foundational ankle draft studies by Liu et al. (2017) and Schiavon et al. (2016), enabling direct comparability. This duration is also consistent with the broader local thermal discomfort literature and exceeds the 15-minute evaluation window specified in ASHRAE Standard 55 for assessing local discomfort conditions.
 To assess the potential effect of longer exposure, we extrapolated the measured lower-leg skin temperature trajectories to 90 minutes using exponential models, and validated these projections against the Advanced Berkeley Comfort (ABC) model, a multi-node transient human thermal model that simulates heat exchange between body segments and the environment over time and has been extensively validated against experimental data (Huizenga et al., 2001). The ABC model predicted an additional lower-leg skin temperature decrease of only 0.3–0.7°C beyond 20 minutes and a corresponding change in whole-body thermal sensation below 0.3 TSV units. We acknowledge that subjective dissatisfaction rates beyond the tested period cannot be directly predicted and may be somewhat higher under sustained exposure; this is discussed in the Limitations section and the relevant passage in the Results has been revised to reflect this uncertainty more explicitly.</t>
+  </si>
+  <si>
+    <t>We thank the reviewer for this suggestion and agree. We have revised the relevant sentence to remove the assertion that the 20-minute duration "is expected to have a limited influence" on the main findings. The revised text retains the ABC model extrapolation as supporting evidence for the conclusion that the main findings are unlikely to be substantially altered, while explicitly acknowledging that subjective dissatisfaction beyond the tested period cannot be directly assessed and may be somewhat higher under prolonged real-office exposure.</t>
+  </si>
+  <si>
+    <t>We thank the reviewer for this comment and are happy to clarify. The proposed model is explicitly intended to predict population-average responses, specifically, the predicted percentage of occupants dissatisfied with ankle draft under given conditions. This follows the same PPD framework established by Fanger and adopted in ASHRAE Standard 55, where the model output by definition represents the expected proportion dissatisfied across a group rather than an individual's response. The considerable scatter visible in Figures 3–6 reflects the well-documented inter-individual variability in local thermal sensitivity, which is also why a mixed-effects model structure was chosen: the random subject intercept explicitly accounts for between-subject heterogeneity, preventing it from inflating the fixed-effect estimates. The low marginal R² values are consistent with this interpretation: the fixed predictors (air speed, thermal sensation) explain the population-level trend, while the remaining variance is largely attributable to individual differences. We have added a brief clarifying statement to the manuscript to make the intended scope of the model explicit.</t>
+  </si>
+  <si>
+    <t>We thank the reviewer for this comment. We note that the foundational ankle draft model of Liu et al. (2017), which underpins the ASHRAE Standard 55 criterion our study seeks to update, was itself derived under purely convective conditions without radiant asymmetry. The comparison between our findings and the existing model is therefore conducted under equivalent boundary conditions, and the central conclusion, that covered-ankle dissatisfaction is substantially lower than predicted, remains valid regardless of radiant asymmetry. Moreover, ASHRAE Standard 55 treats ankle draft and radiant asymmetry as independent local discomfort criteria evaluated in separate sections of the standard; our study addresses the ankle draft criterion specifically. We have added a clarifying sentence to the Implications section noting that the covered-ankle criterion applies to the convective component of window downdraft and that radiant asymmetry should be assessed independently per ASHRAE Standard 55.</t>
+  </si>
+  <si>
+    <t>We thank the reviewer for this comment. We respectfully note that the existing ASHRAE 55 ankle draft model was also derived without radiant asymmetry, so the experimental boundary conditions are equivalent and the relative comparison is valid. ASHRAE Standard 55 evaluates ankle draft and radiant asymmetry as separate, independent criteria. The practical implications discussed in this paper, specifically the potential to relax perimeter heating requirements, relate to the ankle draft component only. Where perimeter heating is additionally required to mitigate radiant asymmetry from cold glazing, this is a separate design consideration unaffected by our findings. We have added a clarifying sentence to the Implications section to make this distinction explicit.</t>
+  </si>
+  <si>
+    <t>We thank the reviewer for this comment. We would like to highlight two points. First, the tested ankle-level conditions (air temperatures of 17–20°C, air speeds of 0.1–0.7 m/s, turbulence intensity of approximately 30%, and rearward airflow direction) were selected to span the range reported for window downdraft in field studies and CFD simulations of typical office perimeter zones (Manz (2004), Lyons (1999)), and to be directly comparable with prior ankle draft studies. The measured ankle-level conditions are reported in Table 3. The airflow direction, from behind toward the lower legs, matches the geometry of window downdraft when workstations face awayfrom the façade, identified by Toftum (1997) as the most thermally sensitive direction.Second, and more fundamentally, the proposed model takes ankle-level air speed, air temperature, and whole-body thermal sensation as inputs — all directly measurable parameters that characterize local airflow conditions regardless of their source. The model is therefore not limited to window downdraft but is equally applicable to other low-velocity air distribution strategies that produce similar ankle-level conditions, such as underfloor air distribution (UFAD) or displacement ventilation systems — the same scenarios for which the original Liu et al. (2017) model was derived. We have added a brief note to the Discussion to clarify this broader applicability.</t>
+  </si>
+  <si>
+    <t>We thank the reviewer for this comment. We have added a simulation-based power analysis to the Methods section (Statistical analysis → Sample size and statistical power). Because no prior data existed for the covered-ankle condition, we used the GL MM fitted to the 88 exposed-ankle participants from Liu et al. (2017) as the reference effect size. This is a conservative choice: the effect of air speed on dissatisfaction is expected to be smaller when ankles are covered, so demonstrating adequate power for the larger exposed-ankle effect constitutes a lower bound on the power available for the covered-ankle comparison. Using the simr package (Green &amp; MacLeod, 2016), we simulated 1,000 datasets at each of seven sample sizes ranging from 10 to 88 and estimated the proportion of simulations in which the fixed effect of ankle air speed was detected at α =0.05. Power reached 80% at N = 30 participants (95% CI: 79.9–84.7%), confirming that our sample of 51 exceeded this threshold by a comfortable margin (power at N = 51: 98.9%, 95% CI: 98.0–99.5%).</t>
+  </si>
+  <si>
+    <t>Requires review by Patrick</t>
   </si>
 </sst>
 </file>
@@ -421,7 +442,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -479,6 +500,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -787,11 +814,11 @@
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="100" customWidth="1"/>
+    <col min="3" max="3" width="64.83203125" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="28.33203125" style="14" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="55.83203125" style="14" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
     <col min="8" max="8" width="80.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -861,7 +888,7 @@
       <c r="F3" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="20" t="s">
         <v>81</v>
       </c>
     </row>
@@ -878,9 +905,15 @@
       <c r="D4" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="E4" s="8"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="8"/>
+      <c r="E4" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>96</v>
+      </c>
       <c r="H4" s="8" t="s">
         <v>58</v>
       </c>
@@ -927,7 +960,7 @@
       <c r="F6" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="21" t="s">
         <v>86</v>
       </c>
     </row>
@@ -992,7 +1025,7 @@
       <c r="F9" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="G9" s="21" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1033,8 +1066,12 @@
       <c r="D11" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="9"/>
+      <c r="E11" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>92</v>
+      </c>
       <c r="G11" s="8"/>
     </row>
     <row r="12" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -1217,8 +1254,12 @@
       <c r="D20" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="E20" s="8"/>
-      <c r="F20" s="9"/>
+      <c r="E20" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>94</v>
+      </c>
       <c r="G20" s="8"/>
       <c r="H20" s="9" t="s">
         <v>61</v>
@@ -1243,7 +1284,9 @@
       <c r="F21" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="G21" s="8"/>
+      <c r="G21" s="21" t="s">
+        <v>86</v>
+      </c>
       <c r="H21" s="9"/>
     </row>
     <row r="22" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
@@ -1259,8 +1302,12 @@
       <c r="D22" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="E22" s="8"/>
-      <c r="F22" s="9"/>
+      <c r="E22" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>90</v>
+      </c>
       <c r="G22" s="8"/>
       <c r="H22" s="9" t="s">
         <v>62</v>
@@ -1301,7 +1348,12 @@
       <c r="D24" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="F24" s="9"/>
+      <c r="E24" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>91</v>
+      </c>
       <c r="G24" s="8"/>
       <c r="H24" s="9" t="s">
         <v>63</v>
@@ -1342,8 +1394,12 @@
       <c r="D26" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="E26" s="8"/>
-      <c r="F26" s="9"/>
+      <c r="E26" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>93</v>
+      </c>
       <c r="G26" s="8"/>
       <c r="H26" s="9"/>
     </row>

</xml_diff>